<commit_message>
update coordinates and things in dashboard
</commit_message>
<xml_diff>
--- a/พิกัดของแต่ละพื้นที่.xlsx
+++ b/พิกัดของแต่ละพื้นที่.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\DSDEad\real_shit\DSDEad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BE0680-C08E-4CD5-83A0-6E10463F4AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC6166FD-56FC-44FE-807D-A4995668D195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7050" yWindow="1620" windowWidth="17550" windowHeight="13815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -487,10 +487,10 @@
         <v>9</v>
       </c>
       <c r="D2">
-        <v>18.591699999999999</v>
+        <v>18.588688999999999</v>
       </c>
       <c r="E2">
-        <v>98.759100000000004</v>
+        <v>98.749458000000004</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -504,10 +504,10 @@
         <v>9</v>
       </c>
       <c r="D3">
-        <v>18.675999999999998</v>
+        <v>18.680264000000001</v>
       </c>
       <c r="E3">
-        <v>98.744</v>
+        <v>98.781912000000005</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -521,10 +521,10 @@
         <v>10</v>
       </c>
       <c r="D4">
-        <v>17.893000000000001</v>
+        <v>17.888123</v>
       </c>
       <c r="E4">
-        <v>98.730500000000006</v>
+        <v>98.701460999999995</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -538,10 +538,10 @@
         <v>10</v>
       </c>
       <c r="D5">
-        <v>17.982299999999999</v>
+        <v>17.918869000000001</v>
       </c>
       <c r="E5">
-        <v>98.688900000000004</v>
+        <v>98.576525000000004</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -555,10 +555,10 @@
         <v>10</v>
       </c>
       <c r="D6">
-        <v>17.982299999999999</v>
+        <v>17.950762999999998</v>
       </c>
       <c r="E6">
-        <v>98.688900000000004</v>
+        <v>98.689145999999994</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -572,10 +572,10 @@
         <v>10</v>
       </c>
       <c r="D7">
-        <v>17.640999999999998</v>
+        <v>18.016069999999999</v>
       </c>
       <c r="E7">
-        <v>98.475999999999999</v>
+        <v>98.660632000000007</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -589,10 +589,10 @@
         <v>10</v>
       </c>
       <c r="D8">
-        <v>17.734000000000002</v>
+        <v>18.053217</v>
       </c>
       <c r="E8">
-        <v>98.512</v>
+        <v>98.624668999999997</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -606,10 +606,10 @@
         <v>10</v>
       </c>
       <c r="D9">
-        <v>17.529</v>
+        <v>17.886451999999998</v>
       </c>
       <c r="E9">
-        <v>98.393000000000001</v>
+        <v>98.787381999999994</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -623,10 +623,10 @@
         <v>10</v>
       </c>
       <c r="D10">
-        <v>17.834800000000001</v>
+        <v>17.837779999999999</v>
       </c>
       <c r="E10">
-        <v>98.594099999999997</v>
+        <v>98.572541000000001</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -640,10 +640,10 @@
         <v>10</v>
       </c>
       <c r="D11">
-        <v>17.393999999999998</v>
+        <v>18.358525</v>
       </c>
       <c r="E11">
-        <v>98.275000000000006</v>
+        <v>98.232825000000005</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -657,10 +657,10 @@
         <v>10</v>
       </c>
       <c r="D12">
-        <v>17.78</v>
+        <v>17.859960000000001</v>
       </c>
       <c r="E12">
-        <v>98.37</v>
+        <v>98.154386000000002</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -674,10 +674,10 @@
         <v>10</v>
       </c>
       <c r="D13">
-        <v>17.45</v>
+        <v>17.423642999999998</v>
       </c>
       <c r="E13">
-        <v>98.31</v>
+        <v>98.504570999999999</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -691,10 +691,10 @@
         <v>10</v>
       </c>
       <c r="D14">
-        <v>17.374700000000001</v>
+        <v>17.397321000000002</v>
       </c>
       <c r="E14">
-        <v>98.374600000000001</v>
+        <v>98.392285999999999</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -708,10 +708,10 @@
         <v>10</v>
       </c>
       <c r="D15">
-        <v>17.565000000000001</v>
+        <v>17.660843</v>
       </c>
       <c r="E15">
-        <v>98.418000000000006</v>
+        <v>98.199990999999997</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -725,10 +725,10 @@
         <v>10</v>
       </c>
       <c r="D16">
-        <v>17.381</v>
+        <v>17.670583000000001</v>
       </c>
       <c r="E16">
-        <v>98.346999999999994</v>
+        <v>98.401596999999995</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -759,10 +759,10 @@
         <v>10</v>
       </c>
       <c r="D18">
-        <v>17.8</v>
+        <v>17.803391999999999</v>
       </c>
       <c r="E18">
-        <v>98.366</v>
+        <v>98.362506999999994</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -776,10 +776,10 @@
         <v>10</v>
       </c>
       <c r="D19">
-        <v>18.04</v>
+        <v>18.010183000000001</v>
       </c>
       <c r="E19">
-        <v>98.34</v>
+        <v>98.516266000000002</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -793,10 +793,10 @@
         <v>10</v>
       </c>
       <c r="D20">
-        <v>18.114999999999998</v>
+        <v>18.158991</v>
       </c>
       <c r="E20">
-        <v>98.28</v>
+        <v>98.231487000000001</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -810,10 +810,10 @@
         <v>10</v>
       </c>
       <c r="D21">
-        <v>18.147777999999999</v>
+        <v>18.153109000000001</v>
       </c>
       <c r="E21">
-        <v>98.348222000000007</v>
+        <v>98.362620000000007</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -827,10 +827,10 @@
         <v>10</v>
       </c>
       <c r="D22">
-        <v>18.052</v>
+        <v>18.105032000000001</v>
       </c>
       <c r="E22">
-        <v>98.456999999999994</v>
+        <v>98.709530000000001</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -844,10 +844,10 @@
         <v>10</v>
       </c>
       <c r="D23">
-        <v>18.108000000000001</v>
+        <v>18.164196</v>
       </c>
       <c r="E23">
-        <v>98.468000000000004</v>
+        <v>98.514455999999996</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -861,10 +861,10 @@
         <v>10</v>
       </c>
       <c r="D24">
-        <v>18.094000000000001</v>
+        <v>18.202231999999999</v>
       </c>
       <c r="E24">
-        <v>98.471999999999994</v>
+        <v>98.598478999999998</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -878,10 +878,10 @@
         <v>10</v>
       </c>
       <c r="D25">
-        <v>18.118444</v>
+        <v>18.171417999999999</v>
       </c>
       <c r="E25">
-        <v>98.603222000000002</v>
+        <v>98.620311999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>